<commit_message>
Update NPV model with CIFR project data from SEC filings
Replaces placeholder projects with verified CIFR numbers:
- Barber Lake: Fluidstack/Google, $3.83B / 10yr NNN, 207 MW critical IT
- Black Pearl: AWS, $5.5B / 15yr NNN, 216 MW critical IT
- Stingray: AWS, ~$2.06B long-term NNN, 70 MW critical IT, $810M project financing
- Colchis / Ulysses / McLennan: pipeline sites with probability-weighted assumptions

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S7tkW9c6aRn5soHaYywQvB
</commit_message>
<xml_diff>
--- a/npv_model.xlsx
+++ b/npv_model.xlsx
@@ -656,7 +656,7 @@
       <c r="A2" s="3" t="n"/>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Base Year: 2026  |  All figures in $mm USD  |  Supports: Colocation (CIFR/WULF) &amp; AI Cloud (IREN)</t>
+          <t>CIFR (Cipher Digital) — 3 Signed Projects + 3 Pipeline Sites  |  Base Year: 2026  |  All figures in $mm USD</t>
         </is>
       </c>
       <c r="C2" s="3" t="n"/>
@@ -740,12 +740,12 @@
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t>Cloud</t>
+          <t>Colo</t>
         </is>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
-          <t>Cloud</t>
+          <t>Colo</t>
         </is>
       </c>
       <c r="J6" s="9" t="inlineStr">
@@ -772,22 +772,22 @@
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>WULF</t>
+          <t>CIFR</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>WULF</t>
+          <t>CIFR</t>
         </is>
       </c>
       <c r="H7" s="8" t="inlineStr">
         <is>
-          <t>IREN</t>
+          <t>CIFR</t>
         </is>
       </c>
       <c r="I7" s="8" t="inlineStr">
         <is>
-          <t>IREN</t>
+          <t>CIFR</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Barber Lake</t>
+          <t>Barber Lake (Fluidstack)</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
@@ -809,22 +809,22 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>Lake Mariner (Core42)</t>
+          <t>Stingray (AWS)</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>Abernathy JV</t>
+          <t>Colchis (W. Texas)</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>NVIDIA Blackwell Contract</t>
+          <t>Ulysses (Ohio)</t>
         </is>
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>Microsoft AI Contract</t>
+          <t>McLennan (Central TX)</t>
         </is>
       </c>
     </row>
@@ -836,32 +836,32 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Under construction; Phase I Sept 2026</t>
+          <t>Signed 10-yr NNN; Fluidstack/Google-backed; Phase I Sep 2026 → full ramp Jan 2027</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>Under construction; AWS 15-yr lease; Phase I Q4 2026</t>
+          <t>Signed 15-yr NNN; Amazon Data Services; Phase I Q4 2026 → full ramp Q1 2027</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>Operational — 60 MW live</t>
+          <t>Signed long-term NNN; Amazon Data Services; earthwork+substation Q1 2026; H1 2026 COD</t>
         </is>
       </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
-          <t>Under construction; Fluidstack/Google; 25-yr lease</t>
+          <t>Pipeline; 1 GW site; majority JV stake; AEP dual interconnect executed; no lease signed</t>
         </is>
       </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>Signed; 20% prepayment received; ramp early 2027</t>
+          <t>Pipeline; site acquired Dec 2025; AEP Ohio / future PJM; Q4 2027 est.</t>
         </is>
       </c>
       <c r="I9" s="11" t="inlineStr">
         <is>
-          <t>Signed; $9.7B total / 5yr; GB300 NVL72</t>
+          <t>Pipeline; option exercised Feb 2026; ERCOT interconnect queue; est. 2028</t>
         </is>
       </c>
     </row>
@@ -890,19 +890,23 @@
         </is>
       </c>
       <c r="D12" s="15" t="n">
-        <v>300</v>
+        <v>207</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>300</v>
+        <v>216</v>
       </c>
       <c r="F12" s="15" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="G12" s="15" t="n">
-        <v>168</v>
-      </c>
-      <c r="H12" s="15" t="n"/>
-      <c r="I12" s="15" t="n"/>
+        <v>500</v>
+      </c>
+      <c r="H12" s="15" t="n">
+        <v>200</v>
+      </c>
+      <c r="I12" s="15" t="n">
+        <v>500</v>
+      </c>
       <c r="J12" s="9" t="inlineStr">
         <is>
           <t>Net MW for colocation; or leave blank for Cloud</t>
@@ -915,20 +919,18 @@
           <t>Revenue per Watt per Year ($/W/yr)</t>
         </is>
       </c>
-      <c r="D13" s="16" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="E13" s="16" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="F13" s="16" t="n">
-        <v>1.65</v>
-      </c>
+      <c r="D13" s="16" t="n"/>
+      <c r="E13" s="16" t="n"/>
+      <c r="F13" s="16" t="n"/>
       <c r="G13" s="16" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="H13" s="16" t="n"/>
-      <c r="I13" s="16" t="n"/>
+        <v>1.5</v>
+      </c>
+      <c r="H13" s="16" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I13" s="16" t="n">
+        <v>1.5</v>
+      </c>
       <c r="J13" s="9" t="inlineStr">
         <is>
           <t>Colo: ~$1.50–1.65/W/yr  |  Cloud: leave blank</t>
@@ -941,16 +943,18 @@
           <t>Contracted ARR ($mm/yr)</t>
         </is>
       </c>
-      <c r="D14" s="17" t="n"/>
-      <c r="E14" s="17" t="n"/>
-      <c r="F14" s="17" t="n"/>
+      <c r="D14" s="17" t="n">
+        <v>383</v>
+      </c>
+      <c r="E14" s="17" t="n">
+        <v>367</v>
+      </c>
+      <c r="F14" s="17" t="n">
+        <v>137</v>
+      </c>
       <c r="G14" s="17" t="n"/>
-      <c r="H14" s="17" t="n">
-        <v>1900</v>
-      </c>
-      <c r="I14" s="17" t="n">
-        <v>1940</v>
-      </c>
+      <c r="H14" s="17" t="n"/>
+      <c r="I14" s="17" t="n"/>
       <c r="J14" s="9" t="inlineStr">
         <is>
           <t>Cloud projects: enter annual contracted revenue here</t>
@@ -1011,10 +1015,10 @@
         <v>1</v>
       </c>
       <c r="H16" s="20" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="I16" s="20" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="J16" s="9" t="inlineStr">
         <is>
@@ -1076,10 +1080,10 @@
         <v>0.85</v>
       </c>
       <c r="H18" s="20" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="I18" s="20" t="n">
-        <v>0.79</v>
+        <v>0.85</v>
       </c>
       <c r="J18" s="9" t="inlineStr">
         <is>
@@ -1146,12 +1150,8 @@
       <c r="E22" s="17" t="n"/>
       <c r="F22" s="17" t="n"/>
       <c r="G22" s="17" t="n"/>
-      <c r="H22" s="17" t="n">
-        <v>180</v>
-      </c>
-      <c r="I22" s="17" t="n">
-        <v>220</v>
-      </c>
+      <c r="H22" s="17" t="n"/>
+      <c r="I22" s="17" t="n"/>
       <c r="J22" s="9" t="inlineStr">
         <is>
           <t>Cloud: est. from MW × $/kWh</t>
@@ -1168,12 +1168,8 @@
       <c r="E23" s="17" t="n"/>
       <c r="F23" s="17" t="n"/>
       <c r="G23" s="17" t="n"/>
-      <c r="H23" s="17" t="n">
-        <v>80</v>
-      </c>
-      <c r="I23" s="17" t="n">
-        <v>100</v>
-      </c>
+      <c r="H23" s="17" t="n"/>
+      <c r="I23" s="17" t="n"/>
       <c r="J23" s="9" t="inlineStr"/>
     </row>
     <row r="24" ht="15" customHeight="1">
@@ -1186,12 +1182,8 @@
       <c r="E24" s="17" t="n"/>
       <c r="F24" s="17" t="n"/>
       <c r="G24" s="17" t="n"/>
-      <c r="H24" s="17" t="n">
-        <v>40</v>
-      </c>
-      <c r="I24" s="17" t="n">
-        <v>50</v>
-      </c>
+      <c r="H24" s="17" t="n"/>
+      <c r="I24" s="17" t="n"/>
       <c r="J24" s="9" t="inlineStr"/>
     </row>
     <row r="25" ht="15" customHeight="1">
@@ -1204,12 +1196,8 @@
       <c r="E25" s="17" t="n"/>
       <c r="F25" s="17" t="n"/>
       <c r="G25" s="17" t="n"/>
-      <c r="H25" s="17" t="n">
-        <v>84</v>
-      </c>
-      <c r="I25" s="17" t="n">
-        <v>105</v>
-      </c>
+      <c r="H25" s="17" t="n"/>
+      <c r="I25" s="17" t="n"/>
       <c r="J25" s="9">
         <f> Debt × Interest Rate</f>
         <v/>
@@ -1315,13 +1303,13 @@
         <v>2026</v>
       </c>
       <c r="G30" s="15" t="n">
-        <v>2027</v>
+        <v>2029</v>
       </c>
       <c r="H30" s="15" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
       <c r="I30" s="15" t="n">
-        <v>2026</v>
+        <v>2028</v>
       </c>
       <c r="J30" s="9" t="inlineStr">
         <is>
@@ -1371,7 +1359,7 @@
         </is>
       </c>
       <c r="D32" s="15" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E32" s="15" t="n">
         <v>15</v>
@@ -1380,13 +1368,13 @@
         <v>15</v>
       </c>
       <c r="G32" s="15" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="H32" s="15" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="I32" s="15" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="J32" s="9" t="inlineStr"/>
     </row>
@@ -1409,10 +1397,10 @@
         <v>0.1</v>
       </c>
       <c r="H33" s="20" t="n">
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
       <c r="I33" s="20" t="n">
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
       <c r="J33" s="9" t="inlineStr">
         <is>
@@ -1511,22 +1499,22 @@
         </is>
       </c>
       <c r="D38" s="17" t="n">
-        <v>450</v>
+        <v>400</v>
       </c>
       <c r="E38" s="17" t="n">
-        <v>450</v>
+        <v>430</v>
       </c>
       <c r="F38" s="17" t="n">
-        <v>0</v>
+        <v>953</v>
       </c>
       <c r="G38" s="17" t="n">
-        <v>252</v>
+        <v>750</v>
       </c>
       <c r="H38" s="17" t="n">
-        <v>2000</v>
+        <v>300</v>
       </c>
       <c r="I38" s="17" t="n">
-        <v>2500</v>
+        <v>750</v>
       </c>
       <c r="J38" s="9" t="inlineStr">
         <is>
@@ -1550,13 +1538,13 @@
         <v>0.85</v>
       </c>
       <c r="G39" s="20" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="H39" s="20" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="I39" s="20" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="J39" s="9" t="inlineStr">
         <is>
@@ -1571,22 +1559,22 @@
         </is>
       </c>
       <c r="D40" s="17" t="n">
-        <v>382.5</v>
+        <v>340</v>
       </c>
       <c r="E40" s="17" t="n">
-        <v>382.5</v>
+        <v>365</v>
       </c>
       <c r="F40" s="17" t="n">
-        <v>0</v>
+        <v>810</v>
       </c>
       <c r="G40" s="17" t="n">
-        <v>214.2</v>
+        <v>600</v>
       </c>
       <c r="H40" s="17" t="n">
-        <v>1200</v>
+        <v>240</v>
       </c>
       <c r="I40" s="17" t="n">
-        <v>1500</v>
+        <v>600</v>
       </c>
       <c r="J40" s="9" t="inlineStr">
         <is>
@@ -1653,12 +1641,8 @@
       <c r="E44" s="15" t="n"/>
       <c r="F44" s="15" t="n"/>
       <c r="G44" s="15" t="n"/>
-      <c r="H44" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="I44" s="15" t="n">
-        <v>4</v>
-      </c>
+      <c r="H44" s="15" t="n"/>
+      <c r="I44" s="15" t="n"/>
       <c r="J44" s="9" t="inlineStr">
         <is>
           <t>Typically 4 years for Blackwell-class</t>
@@ -1675,12 +1659,8 @@
       <c r="E45" s="20" t="n"/>
       <c r="F45" s="20" t="n"/>
       <c r="G45" s="20" t="n"/>
-      <c r="H45" s="20" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="I45" s="20" t="n">
-        <v>0.8</v>
-      </c>
+      <c r="H45" s="20" t="n"/>
+      <c r="I45" s="20" t="n"/>
       <c r="J45" s="9" t="inlineStr">
         <is>
           <t>~80% — next-gen GPUs cost similar</t>
@@ -1823,13 +1803,13 @@
         <v>5</v>
       </c>
       <c r="G51" s="15" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H51" s="15" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I51" s="15" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J51" s="9" t="inlineStr">
         <is>
@@ -1853,13 +1833,13 @@
         <v>0.9</v>
       </c>
       <c r="G52" s="20" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="H52" s="20" t="n">
-        <v>0.75</v>
+        <v>0.85</v>
       </c>
       <c r="I52" s="20" t="n">
-        <v>0.75</v>
+        <v>0.85</v>
       </c>
       <c r="J52" s="9" t="inlineStr">
         <is>
@@ -1874,22 +1854,22 @@
         </is>
       </c>
       <c r="D53" s="20" t="n">
-        <v>0.6</v>
+        <v>0.65</v>
       </c>
       <c r="E53" s="20" t="n">
-        <v>0.6</v>
+        <v>0.65</v>
       </c>
       <c r="F53" s="20" t="n">
-        <v>0.6</v>
+        <v>0.65</v>
       </c>
       <c r="G53" s="20" t="n">
-        <v>0</v>
+        <v>0.55</v>
       </c>
       <c r="H53" s="20" t="n">
-        <v>0.5</v>
+        <v>0.55</v>
       </c>
       <c r="I53" s="20" t="n">
-        <v>0.5</v>
+        <v>0.55</v>
       </c>
       <c r="J53" s="9" t="inlineStr"/>
     </row>
@@ -1958,13 +1938,13 @@
         <v>1</v>
       </c>
       <c r="G57" s="20" t="n">
-        <v>1</v>
+        <v>0.35</v>
       </c>
       <c r="H57" s="20" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="I57" s="20" t="n">
-        <v>1</v>
+        <v>0.35</v>
       </c>
       <c r="J57" s="9" t="inlineStr">
         <is>
@@ -1979,22 +1959,22 @@
         </is>
       </c>
       <c r="D58" s="20" t="n">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
       <c r="E58" s="20" t="n">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
       <c r="F58" s="20" t="n">
-        <v>1</v>
+        <v>0.92</v>
       </c>
       <c r="G58" s="20" t="n">
-        <v>0.8</v>
+        <v>0.75</v>
       </c>
       <c r="H58" s="20" t="n">
-        <v>0.85</v>
+        <v>0.78</v>
       </c>
       <c r="I58" s="20" t="n">
-        <v>0.9</v>
+        <v>0.75</v>
       </c>
       <c r="J58" s="9" t="inlineStr">
         <is>

</xml_diff>